<commit_message>
chore(deps): update the dev dependencies
Update TypeScript to 7, Vitest to 5 and @types/node to 26, and apply the
format of Prettier 3.9. Regenerate the examples: write-excel-file 4.1
writes the attributes of the sheet element in a different order.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AXig7iCj3NkYjt6HYrt5WE
</commit_message>
<xml_diff>
--- a/examples/list-range-cross-sheet.xlsx
+++ b/examples/list-range-cross-sheet.xlsx
@@ -6,8 +6,8 @@
     <workbookView/>
   </bookViews>
   <sheets>
-    <sheet name="Main" sheetId="1" r:id="rId1"/>
-    <sheet name="Lists" sheetId="2" r:id="rId2"/>
+    <sheet r:id="rId1" sheetId="1" name="Main"/>
+    <sheet r:id="rId2" sheetId="2" name="Lists"/>
   </sheets>
   <definedNames/>
   <calcPr/>

</xml_diff>